<commit_message>
Memory map updated (KIM-1 IO)
</commit_message>
<xml_diff>
--- a/Manuals/R65 OS Memory Map.xlsx
+++ b/Manuals/R65 OS Memory Map.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11020"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rricharz/Projects/R65/Manuals/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D99FC8C-4328-604B-962A-1E4C4161367E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{123F169E-135C-8544-8805-794E6BD9269B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5580" yWindow="620" windowWidth="19120" windowHeight="16760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5580" yWindow="620" windowWidth="21780" windowHeight="16760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="memory map" sheetId="1" r:id="rId1"/>
     <sheet name="notes" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'memory map'!$A$1:$H$160</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'memory map'!$A$1:$H$167</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'memory map'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="0"/>
@@ -87,7 +87,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1001" uniqueCount="525">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1044" uniqueCount="554">
   <si>
     <t>zone</t>
   </si>
@@ -1662,6 +1662,93 @@
   </si>
   <si>
     <t>25 bytes</t>
+  </si>
+  <si>
+    <t>HOSTOUT</t>
+  </si>
+  <si>
+    <t>1700-177f</t>
+  </si>
+  <si>
+    <t>I/O</t>
+  </si>
+  <si>
+    <t>1702</t>
+  </si>
+  <si>
+    <t>USPBD / D8_USPBD</t>
+  </si>
+  <si>
+    <t>iocontrol,emulator</t>
+  </si>
+  <si>
+    <t>Existing user-port B data register; LED display</t>
+  </si>
+  <si>
+    <t>1703</t>
+  </si>
+  <si>
+    <t>USPBDD</t>
+  </si>
+  <si>
+    <t>iocontrol</t>
+  </si>
+  <si>
+    <t>User-port B data-direction register</t>
+  </si>
+  <si>
+    <t>1708</t>
+  </si>
+  <si>
+    <t>KIM_MOUSEMODE</t>
+  </si>
+  <si>
+    <t>emulator,Pascal</t>
+  </si>
+  <si>
+    <t>Mouse event: 0 none, 1 text, 2 graphics</t>
+  </si>
+  <si>
+    <t>Reading mode freezes event until mouse Y is read</t>
+  </si>
+  <si>
+    <t>1709</t>
+  </si>
+  <si>
+    <t>KIM_MOUSEX</t>
+  </si>
+  <si>
+    <t>Mouse X: text column 0–47 or graphics X 0–223</t>
+  </si>
+  <si>
+    <t>Read after mouse mode</t>
+  </si>
+  <si>
+    <t>170a</t>
+  </si>
+  <si>
+    <t>KIM_MOUSEY</t>
+  </si>
+  <si>
+    <t>Mouse Y: text row 0–15 or graphics Y 0–117</t>
+  </si>
+  <si>
+    <t>Reading Y clears event and releases freeze</t>
+  </si>
+  <si>
+    <t>1747</t>
+  </si>
+  <si>
+    <t>TMSEC / TIMER1 / R8_TMSEC</t>
+  </si>
+  <si>
+    <t>crt,iocontrol,emulator</t>
+  </si>
+  <si>
+    <t>Legacy KIM timer: each read delays ~1 ms and decrements modulo 256</t>
+  </si>
+  <si>
+    <t>Wraparound is required by sound/BEL and delay loops (BPL waits for bit 7)</t>
   </si>
 </sst>
 </file>
@@ -2048,7 +2135,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H162"/>
+  <dimension ref="A1:H169"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="12"/>
   <cols>
     <col min="1" max="1" width="9.5" style="4" customWidth="1"/>
@@ -2058,7 +2145,7 @@
     <col min="5" max="5" width="12" style="4" customWidth="1"/>
     <col min="6" max="6" width="18" style="4" customWidth="1"/>
     <col min="7" max="7" width="9.5" style="4" customWidth="1"/>
-    <col min="8" max="8" width="14" style="4" customWidth="1"/>
+    <col min="8" max="8" width="21.83203125" style="4" customWidth="1"/>
     <col min="9" max="16384" width="8.83203125" style="4"/>
   </cols>
   <sheetData>
@@ -5023,235 +5110,225 @@
       <c r="H123" s="5"/>
     </row>
     <row r="124" spans="1:8" ht="32" customHeight="1">
-      <c r="A124" s="6" t="s">
-        <v>506</v>
-      </c>
-      <c r="B124" s="6" t="s">
-        <v>367</v>
-      </c>
-      <c r="C124" s="6">
-        <v>1</v>
-      </c>
-      <c r="D124" s="6" t="s">
-        <v>368</v>
-      </c>
-      <c r="E124" s="6" t="s">
-        <v>369</v>
-      </c>
-      <c r="F124" s="6" t="s">
-        <v>370</v>
-      </c>
-      <c r="G124" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="H124" s="6"/>
-    </row>
-    <row r="125" spans="1:8" ht="44" customHeight="1">
-      <c r="A125" s="6" t="s">
-        <v>506</v>
+      <c r="A124" s="5" t="s">
+        <v>526</v>
+      </c>
+      <c r="B124" s="5">
+        <v>1700</v>
+      </c>
+      <c r="C124" s="5">
+        <v>1</v>
+      </c>
+      <c r="D124" s="5" t="s">
+        <v>525</v>
+      </c>
+      <c r="E124" s="5" t="s">
+        <v>512</v>
+      </c>
+      <c r="F124" s="5"/>
+      <c r="G124" s="5"/>
+      <c r="H124" s="5"/>
+    </row>
+    <row r="125" spans="1:8" ht="32" customHeight="1">
+      <c r="A125" s="5" t="s">
+        <v>526</v>
       </c>
       <c r="B125" s="5" t="s">
-        <v>371</v>
+        <v>528</v>
       </c>
       <c r="C125" s="5">
         <v>1</v>
       </c>
       <c r="D125" s="5" t="s">
-        <v>372</v>
+        <v>529</v>
       </c>
       <c r="E125" s="5" t="s">
-        <v>373</v>
+        <v>530</v>
       </c>
       <c r="F125" s="5" t="s">
-        <v>374</v>
+        <v>531</v>
       </c>
       <c r="G125" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="H125" s="5" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="126" spans="1:8" ht="68" customHeight="1">
-      <c r="A126" s="6" t="s">
-        <v>506</v>
+        <v>527</v>
+      </c>
+      <c r="H125" s="5"/>
+    </row>
+    <row r="126" spans="1:8" ht="32" customHeight="1">
+      <c r="A126" s="5" t="s">
+        <v>526</v>
       </c>
       <c r="B126" s="5" t="s">
-        <v>375</v>
+        <v>532</v>
       </c>
       <c r="C126" s="5">
         <v>1</v>
       </c>
       <c r="D126" s="5" t="s">
-        <v>376</v>
+        <v>533</v>
       </c>
       <c r="E126" s="5" t="s">
-        <v>140</v>
+        <v>534</v>
       </c>
       <c r="F126" s="5" t="s">
-        <v>377</v>
+        <v>535</v>
       </c>
       <c r="G126" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="H126" s="5" t="s">
-        <v>378</v>
-      </c>
-    </row>
-    <row r="127" spans="1:8" ht="68" customHeight="1">
-      <c r="A127" s="6" t="s">
-        <v>506</v>
+        <v>527</v>
+      </c>
+      <c r="H126" s="5"/>
+    </row>
+    <row r="127" spans="1:8" ht="32" customHeight="1">
+      <c r="A127" s="5" t="s">
+        <v>526</v>
       </c>
       <c r="B127" s="5" t="s">
-        <v>379</v>
+        <v>536</v>
       </c>
       <c r="C127" s="5">
         <v>1</v>
       </c>
       <c r="D127" s="5" t="s">
-        <v>380</v>
+        <v>537</v>
       </c>
       <c r="E127" s="5" t="s">
-        <v>140</v>
+        <v>538</v>
       </c>
       <c r="F127" s="5" t="s">
-        <v>381</v>
+        <v>539</v>
       </c>
       <c r="G127" s="5" t="s">
-        <v>100</v>
+        <v>527</v>
       </c>
       <c r="H127" s="5" t="s">
-        <v>382</v>
-      </c>
-    </row>
-    <row r="128" spans="1:8" ht="68" customHeight="1">
-      <c r="A128" s="6" t="s">
-        <v>506</v>
+        <v>540</v>
+      </c>
+    </row>
+    <row r="128" spans="1:8" ht="32" customHeight="1">
+      <c r="A128" s="5" t="s">
+        <v>526</v>
       </c>
       <c r="B128" s="5" t="s">
-        <v>383</v>
+        <v>541</v>
       </c>
       <c r="C128" s="5">
         <v>1</v>
       </c>
       <c r="D128" s="5" t="s">
-        <v>384</v>
+        <v>542</v>
       </c>
       <c r="E128" s="5" t="s">
-        <v>140</v>
+        <v>538</v>
       </c>
       <c r="F128" s="5" t="s">
-        <v>385</v>
+        <v>543</v>
       </c>
       <c r="G128" s="5" t="s">
-        <v>100</v>
+        <v>527</v>
       </c>
       <c r="H128" s="5" t="s">
-        <v>386</v>
-      </c>
-    </row>
-    <row r="129" spans="1:8" ht="68" customHeight="1">
-      <c r="A129" s="6" t="s">
-        <v>506</v>
+        <v>544</v>
+      </c>
+    </row>
+    <row r="129" spans="1:8" ht="32" customHeight="1">
+      <c r="A129" s="5" t="s">
+        <v>526</v>
       </c>
       <c r="B129" s="5" t="s">
-        <v>387</v>
+        <v>545</v>
       </c>
       <c r="C129" s="5">
         <v>1</v>
       </c>
       <c r="D129" s="5" t="s">
-        <v>388</v>
+        <v>546</v>
       </c>
       <c r="E129" s="5" t="s">
-        <v>140</v>
+        <v>538</v>
       </c>
       <c r="F129" s="5" t="s">
-        <v>389</v>
+        <v>547</v>
       </c>
       <c r="G129" s="5" t="s">
-        <v>100</v>
+        <v>527</v>
       </c>
       <c r="H129" s="5" t="s">
-        <v>390</v>
-      </c>
-    </row>
-    <row r="130" spans="1:8" ht="68" customHeight="1">
-      <c r="A130" s="6" t="s">
-        <v>506</v>
+        <v>548</v>
+      </c>
+    </row>
+    <row r="130" spans="1:8" ht="32" customHeight="1">
+      <c r="A130" s="5" t="s">
+        <v>526</v>
       </c>
       <c r="B130" s="5" t="s">
-        <v>391</v>
+        <v>549</v>
       </c>
       <c r="C130" s="5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D130" s="5" t="s">
-        <v>392</v>
+        <v>550</v>
       </c>
       <c r="E130" s="5" t="s">
-        <v>140</v>
+        <v>551</v>
       </c>
       <c r="F130" s="5" t="s">
-        <v>393</v>
+        <v>552</v>
       </c>
       <c r="G130" s="5" t="s">
-        <v>100</v>
+        <v>527</v>
       </c>
       <c r="H130" s="5" t="s">
-        <v>394</v>
-      </c>
-    </row>
-    <row r="131" spans="1:8" ht="68" customHeight="1">
+        <v>553</v>
+      </c>
+    </row>
+    <row r="131" spans="1:8" ht="32" customHeight="1">
       <c r="A131" s="6" t="s">
         <v>506</v>
       </c>
-      <c r="B131" s="5" t="s">
-        <v>395</v>
-      </c>
-      <c r="C131" s="5">
-        <v>1</v>
-      </c>
-      <c r="D131" s="5" t="s">
-        <v>396</v>
-      </c>
-      <c r="E131" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="F131" s="5" t="s">
-        <v>397</v>
-      </c>
-      <c r="G131" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="H131" s="5" t="s">
-        <v>398</v>
-      </c>
-    </row>
-    <row r="132" spans="1:8" ht="80" customHeight="1">
+      <c r="B131" s="6" t="s">
+        <v>367</v>
+      </c>
+      <c r="C131" s="6">
+        <v>1</v>
+      </c>
+      <c r="D131" s="6" t="s">
+        <v>368</v>
+      </c>
+      <c r="E131" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="F131" s="6" t="s">
+        <v>370</v>
+      </c>
+      <c r="G131" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="H131" s="6"/>
+    </row>
+    <row r="132" spans="1:8" ht="44" customHeight="1">
       <c r="A132" s="6" t="s">
         <v>506</v>
       </c>
       <c r="B132" s="5" t="s">
-        <v>399</v>
+        <v>371</v>
       </c>
       <c r="C132" s="5">
         <v>1</v>
       </c>
       <c r="D132" s="5" t="s">
-        <v>400</v>
+        <v>372</v>
       </c>
       <c r="E132" s="5" t="s">
-        <v>401</v>
+        <v>373</v>
       </c>
       <c r="F132" s="5" t="s">
-        <v>402</v>
+        <v>374</v>
       </c>
       <c r="G132" s="5" t="s">
-        <v>100</v>
+        <v>88</v>
       </c>
       <c r="H132" s="5" t="s">
-        <v>403</v>
+        <v>89</v>
       </c>
     </row>
     <row r="133" spans="1:8" ht="68" customHeight="1">
@@ -5259,25 +5336,25 @@
         <v>506</v>
       </c>
       <c r="B133" s="5" t="s">
-        <v>404</v>
+        <v>375</v>
       </c>
       <c r="C133" s="5">
         <v>1</v>
       </c>
       <c r="D133" s="5" t="s">
-        <v>405</v>
+        <v>376</v>
       </c>
       <c r="E133" s="5" t="s">
         <v>140</v>
       </c>
       <c r="F133" s="5" t="s">
-        <v>406</v>
+        <v>377</v>
       </c>
       <c r="G133" s="5" t="s">
         <v>100</v>
       </c>
       <c r="H133" s="5" t="s">
-        <v>407</v>
+        <v>378</v>
       </c>
     </row>
     <row r="134" spans="1:8" ht="68" customHeight="1">
@@ -5285,25 +5362,25 @@
         <v>506</v>
       </c>
       <c r="B134" s="5" t="s">
-        <v>408</v>
+        <v>379</v>
       </c>
       <c r="C134" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D134" s="5" t="s">
-        <v>409</v>
+        <v>380</v>
       </c>
       <c r="E134" s="5" t="s">
         <v>140</v>
       </c>
       <c r="F134" s="5" t="s">
-        <v>410</v>
+        <v>381</v>
       </c>
       <c r="G134" s="5" t="s">
         <v>100</v>
       </c>
       <c r="H134" s="5" t="s">
-        <v>411</v>
+        <v>382</v>
       </c>
     </row>
     <row r="135" spans="1:8" ht="68" customHeight="1">
@@ -5311,25 +5388,25 @@
         <v>506</v>
       </c>
       <c r="B135" s="5" t="s">
-        <v>412</v>
+        <v>383</v>
       </c>
       <c r="C135" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D135" s="5" t="s">
-        <v>413</v>
+        <v>384</v>
       </c>
       <c r="E135" s="5" t="s">
         <v>140</v>
       </c>
       <c r="F135" s="5" t="s">
-        <v>414</v>
+        <v>385</v>
       </c>
       <c r="G135" s="5" t="s">
         <v>100</v>
       </c>
       <c r="H135" s="5" t="s">
-        <v>415</v>
+        <v>386</v>
       </c>
     </row>
     <row r="136" spans="1:8" ht="68" customHeight="1">
@@ -5337,25 +5414,25 @@
         <v>506</v>
       </c>
       <c r="B136" s="5" t="s">
-        <v>416</v>
+        <v>387</v>
       </c>
       <c r="C136" s="5">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="D136" s="5" t="s">
-        <v>417</v>
+        <v>388</v>
       </c>
       <c r="E136" s="5" t="s">
         <v>140</v>
       </c>
       <c r="F136" s="5" t="s">
-        <v>418</v>
+        <v>389</v>
       </c>
       <c r="G136" s="5" t="s">
         <v>100</v>
       </c>
       <c r="H136" s="5" t="s">
-        <v>419</v>
+        <v>390</v>
       </c>
     </row>
     <row r="137" spans="1:8" ht="68" customHeight="1">
@@ -5363,207 +5440,207 @@
         <v>506</v>
       </c>
       <c r="B137" s="5" t="s">
-        <v>420</v>
+        <v>391</v>
       </c>
       <c r="C137" s="5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D137" s="5" t="s">
-        <v>421</v>
+        <v>392</v>
       </c>
       <c r="E137" s="5" t="s">
         <v>140</v>
       </c>
       <c r="F137" s="5" t="s">
-        <v>422</v>
+        <v>393</v>
       </c>
       <c r="G137" s="5" t="s">
         <v>100</v>
       </c>
       <c r="H137" s="5" t="s">
-        <v>423</v>
-      </c>
-    </row>
-    <row r="138" spans="1:8" ht="44" customHeight="1">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="138" spans="1:8" ht="68" customHeight="1">
       <c r="A138" s="6" t="s">
         <v>506</v>
       </c>
       <c r="B138" s="5" t="s">
-        <v>424</v>
+        <v>395</v>
       </c>
       <c r="C138" s="5">
         <v>1</v>
       </c>
       <c r="D138" s="5" t="s">
-        <v>425</v>
+        <v>396</v>
       </c>
       <c r="E138" s="5" t="s">
-        <v>160</v>
+        <v>140</v>
       </c>
       <c r="F138" s="5" t="s">
-        <v>426</v>
+        <v>397</v>
       </c>
       <c r="G138" s="5" t="s">
         <v>100</v>
       </c>
       <c r="H138" s="5" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="139" spans="1:8" ht="44" customHeight="1">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="139" spans="1:8" ht="80" customHeight="1">
       <c r="A139" s="6" t="s">
         <v>506</v>
       </c>
       <c r="B139" s="5" t="s">
-        <v>428</v>
+        <v>399</v>
       </c>
       <c r="C139" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D139" s="5" t="s">
-        <v>429</v>
+        <v>400</v>
       </c>
       <c r="E139" s="5" t="s">
-        <v>160</v>
+        <v>401</v>
       </c>
       <c r="F139" s="5" t="s">
-        <v>430</v>
+        <v>402</v>
       </c>
       <c r="G139" s="5" t="s">
         <v>100</v>
       </c>
       <c r="H139" s="5" t="s">
-        <v>431</v>
-      </c>
-    </row>
-    <row r="140" spans="1:8" ht="44" customHeight="1">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="140" spans="1:8" ht="68" customHeight="1">
       <c r="A140" s="6" t="s">
         <v>506</v>
       </c>
       <c r="B140" s="5" t="s">
-        <v>432</v>
+        <v>404</v>
       </c>
       <c r="C140" s="5">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="D140" s="5" t="s">
-        <v>433</v>
+        <v>405</v>
       </c>
       <c r="E140" s="5" t="s">
-        <v>160</v>
+        <v>140</v>
       </c>
       <c r="F140" s="5" t="s">
-        <v>434</v>
+        <v>406</v>
       </c>
       <c r="G140" s="5" t="s">
         <v>100</v>
       </c>
       <c r="H140" s="5" t="s">
-        <v>435</v>
-      </c>
-    </row>
-    <row r="141" spans="1:8" ht="44" customHeight="1">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="141" spans="1:8" ht="68" customHeight="1">
       <c r="A141" s="6" t="s">
         <v>506</v>
       </c>
       <c r="B141" s="5" t="s">
-        <v>436</v>
+        <v>408</v>
       </c>
       <c r="C141" s="5">
         <v>2</v>
       </c>
       <c r="D141" s="5" t="s">
-        <v>437</v>
+        <v>409</v>
       </c>
       <c r="E141" s="5" t="s">
-        <v>160</v>
+        <v>140</v>
       </c>
       <c r="F141" s="5" t="s">
-        <v>438</v>
+        <v>410</v>
       </c>
       <c r="G141" s="5" t="s">
         <v>100</v>
       </c>
       <c r="H141" s="5" t="s">
-        <v>439</v>
-      </c>
-    </row>
-    <row r="142" spans="1:8" ht="44" customHeight="1">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="142" spans="1:8" ht="68" customHeight="1">
       <c r="A142" s="6" t="s">
         <v>506</v>
       </c>
       <c r="B142" s="5" t="s">
-        <v>440</v>
+        <v>412</v>
       </c>
       <c r="C142" s="5">
         <v>2</v>
       </c>
       <c r="D142" s="5" t="s">
-        <v>441</v>
+        <v>413</v>
       </c>
       <c r="E142" s="5" t="s">
-        <v>160</v>
+        <v>140</v>
       </c>
       <c r="F142" s="5" t="s">
-        <v>442</v>
+        <v>414</v>
       </c>
       <c r="G142" s="5" t="s">
         <v>100</v>
       </c>
       <c r="H142" s="5" t="s">
-        <v>443</v>
-      </c>
-    </row>
-    <row r="143" spans="1:8" ht="44" customHeight="1">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="143" spans="1:8" ht="68" customHeight="1">
       <c r="A143" s="6" t="s">
         <v>506</v>
       </c>
       <c r="B143" s="5" t="s">
-        <v>444</v>
+        <v>416</v>
       </c>
       <c r="C143" s="5">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="D143" s="5" t="s">
-        <v>445</v>
+        <v>417</v>
       </c>
       <c r="E143" s="5" t="s">
-        <v>160</v>
+        <v>140</v>
       </c>
       <c r="F143" s="5" t="s">
-        <v>446</v>
+        <v>418</v>
       </c>
       <c r="G143" s="5" t="s">
         <v>100</v>
       </c>
       <c r="H143" s="5" t="s">
-        <v>447</v>
-      </c>
-    </row>
-    <row r="144" spans="1:8" ht="44" customHeight="1">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="144" spans="1:8" ht="68" customHeight="1">
       <c r="A144" s="6" t="s">
         <v>506</v>
       </c>
       <c r="B144" s="5" t="s">
-        <v>448</v>
+        <v>420</v>
       </c>
       <c r="C144" s="5">
         <v>1</v>
       </c>
       <c r="D144" s="5" t="s">
-        <v>449</v>
+        <v>421</v>
       </c>
       <c r="E144" s="5" t="s">
-        <v>160</v>
+        <v>140</v>
       </c>
       <c r="F144" s="5" t="s">
-        <v>450</v>
+        <v>422</v>
       </c>
       <c r="G144" s="5" t="s">
         <v>100</v>
       </c>
       <c r="H144" s="5" t="s">
-        <v>451</v>
+        <v>423</v>
       </c>
     </row>
     <row r="145" spans="1:8" ht="44" customHeight="1">
@@ -5571,25 +5648,25 @@
         <v>506</v>
       </c>
       <c r="B145" s="5" t="s">
-        <v>452</v>
+        <v>424</v>
       </c>
       <c r="C145" s="5">
         <v>1</v>
       </c>
       <c r="D145" s="5" t="s">
-        <v>453</v>
+        <v>425</v>
       </c>
       <c r="E145" s="5" t="s">
         <v>160</v>
       </c>
       <c r="F145" s="5" t="s">
-        <v>454</v>
+        <v>426</v>
       </c>
       <c r="G145" s="5" t="s">
         <v>100</v>
       </c>
       <c r="H145" s="5" t="s">
-        <v>455</v>
+        <v>427</v>
       </c>
     </row>
     <row r="146" spans="1:8" ht="44" customHeight="1">
@@ -5597,25 +5674,25 @@
         <v>506</v>
       </c>
       <c r="B146" s="5" t="s">
-        <v>456</v>
+        <v>428</v>
       </c>
       <c r="C146" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D146" s="5" t="s">
-        <v>457</v>
+        <v>429</v>
       </c>
       <c r="E146" s="5" t="s">
         <v>160</v>
       </c>
       <c r="F146" s="5" t="s">
-        <v>458</v>
+        <v>430</v>
       </c>
       <c r="G146" s="5" t="s">
         <v>100</v>
       </c>
       <c r="H146" s="5" t="s">
-        <v>459</v>
+        <v>431</v>
       </c>
     </row>
     <row r="147" spans="1:8" ht="44" customHeight="1">
@@ -5623,25 +5700,25 @@
         <v>506</v>
       </c>
       <c r="B147" s="5" t="s">
-        <v>460</v>
+        <v>432</v>
       </c>
       <c r="C147" s="5">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="D147" s="5" t="s">
-        <v>461</v>
+        <v>433</v>
       </c>
       <c r="E147" s="5" t="s">
         <v>160</v>
       </c>
       <c r="F147" s="5" t="s">
-        <v>462</v>
+        <v>434</v>
       </c>
       <c r="G147" s="5" t="s">
         <v>100</v>
       </c>
       <c r="H147" s="5" t="s">
-        <v>463</v>
+        <v>435</v>
       </c>
     </row>
     <row r="148" spans="1:8" ht="44" customHeight="1">
@@ -5649,329 +5726,511 @@
         <v>506</v>
       </c>
       <c r="B148" s="5" t="s">
-        <v>464</v>
+        <v>436</v>
       </c>
       <c r="C148" s="5">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D148" s="5" t="s">
-        <v>465</v>
+        <v>437</v>
       </c>
       <c r="E148" s="5" t="s">
         <v>160</v>
       </c>
       <c r="F148" s="5" t="s">
-        <v>466</v>
+        <v>438</v>
       </c>
       <c r="G148" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="H148" s="5"/>
-    </row>
-    <row r="149" spans="1:8" ht="20" customHeight="1">
+        <v>100</v>
+      </c>
+      <c r="H148" s="5" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="149" spans="1:8" ht="44" customHeight="1">
       <c r="A149" s="6" t="s">
         <v>506</v>
       </c>
       <c r="B149" s="5" t="s">
-        <v>467</v>
+        <v>440</v>
       </c>
       <c r="C149" s="5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D149" s="5" t="s">
-        <v>468</v>
+        <v>441</v>
       </c>
       <c r="E149" s="5" t="s">
         <v>160</v>
       </c>
       <c r="F149" s="5" t="s">
-        <v>469</v>
+        <v>442</v>
       </c>
       <c r="G149" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="H149" s="5"/>
-    </row>
-    <row r="150" spans="1:8" ht="32" customHeight="1">
+        <v>100</v>
+      </c>
+      <c r="H149" s="5" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="150" spans="1:8" ht="44" customHeight="1">
       <c r="A150" s="6" t="s">
         <v>506</v>
       </c>
       <c r="B150" s="5" t="s">
-        <v>470</v>
+        <v>444</v>
       </c>
       <c r="C150" s="5">
         <v>1</v>
       </c>
       <c r="D150" s="5" t="s">
-        <v>471</v>
+        <v>445</v>
       </c>
       <c r="E150" s="5" t="s">
-        <v>472</v>
+        <v>160</v>
       </c>
       <c r="F150" s="5" t="s">
-        <v>473</v>
+        <v>446</v>
       </c>
       <c r="G150" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="H150" s="5"/>
-    </row>
-    <row r="151" spans="1:8" ht="32" customHeight="1">
+        <v>100</v>
+      </c>
+      <c r="H150" s="5" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="151" spans="1:8" ht="44" customHeight="1">
       <c r="A151" s="6" t="s">
         <v>506</v>
       </c>
       <c r="B151" s="5" t="s">
-        <v>474</v>
+        <v>448</v>
       </c>
       <c r="C151" s="5">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="D151" s="5" t="s">
-        <v>475</v>
+        <v>449</v>
       </c>
       <c r="E151" s="5" t="s">
-        <v>472</v>
+        <v>160</v>
       </c>
       <c r="F151" s="5" t="s">
-        <v>476</v>
+        <v>450</v>
       </c>
       <c r="G151" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="H151" s="5"/>
-    </row>
-    <row r="152" spans="1:8" ht="32" customHeight="1">
+        <v>100</v>
+      </c>
+      <c r="H151" s="5" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="152" spans="1:8" ht="44" customHeight="1">
       <c r="A152" s="6" t="s">
         <v>506</v>
       </c>
       <c r="B152" s="5" t="s">
-        <v>477</v>
+        <v>452</v>
       </c>
       <c r="C152" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D152" s="5" t="s">
-        <v>478</v>
+        <v>453</v>
       </c>
       <c r="E152" s="5" t="s">
-        <v>479</v>
+        <v>160</v>
       </c>
       <c r="F152" s="5" t="s">
-        <v>480</v>
+        <v>454</v>
       </c>
       <c r="G152" s="5" t="s">
-        <v>88</v>
+        <v>100</v>
       </c>
       <c r="H152" s="5" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="153" spans="1:8" ht="32" customHeight="1">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="153" spans="1:8" ht="44" customHeight="1">
       <c r="A153" s="6" t="s">
         <v>506</v>
       </c>
       <c r="B153" s="5" t="s">
+        <v>456</v>
+      </c>
+      <c r="C153" s="5">
+        <v>1</v>
+      </c>
+      <c r="D153" s="5" t="s">
+        <v>457</v>
+      </c>
+      <c r="E153" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="F153" s="5" t="s">
+        <v>458</v>
+      </c>
+      <c r="G153" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="H153" s="5" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="154" spans="1:8" ht="44" customHeight="1">
+      <c r="A154" s="6" t="s">
+        <v>506</v>
+      </c>
+      <c r="B154" s="5" t="s">
+        <v>460</v>
+      </c>
+      <c r="C154" s="5">
+        <v>1</v>
+      </c>
+      <c r="D154" s="5" t="s">
+        <v>461</v>
+      </c>
+      <c r="E154" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="F154" s="5" t="s">
+        <v>462</v>
+      </c>
+      <c r="G154" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="H154" s="5" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="155" spans="1:8" ht="44" customHeight="1">
+      <c r="A155" s="6" t="s">
+        <v>506</v>
+      </c>
+      <c r="B155" s="5" t="s">
+        <v>464</v>
+      </c>
+      <c r="C155" s="5">
+        <v>4</v>
+      </c>
+      <c r="D155" s="5" t="s">
+        <v>465</v>
+      </c>
+      <c r="E155" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="F155" s="5" t="s">
+        <v>466</v>
+      </c>
+      <c r="G155" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="H155" s="5"/>
+    </row>
+    <row r="156" spans="1:8" ht="20" customHeight="1">
+      <c r="A156" s="6" t="s">
+        <v>506</v>
+      </c>
+      <c r="B156" s="5" t="s">
+        <v>467</v>
+      </c>
+      <c r="C156" s="5">
+        <v>3</v>
+      </c>
+      <c r="D156" s="5" t="s">
+        <v>468</v>
+      </c>
+      <c r="E156" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="F156" s="5" t="s">
+        <v>469</v>
+      </c>
+      <c r="G156" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="H156" s="5"/>
+    </row>
+    <row r="157" spans="1:8" ht="32" customHeight="1">
+      <c r="A157" s="6" t="s">
+        <v>506</v>
+      </c>
+      <c r="B157" s="5" t="s">
+        <v>470</v>
+      </c>
+      <c r="C157" s="5">
+        <v>1</v>
+      </c>
+      <c r="D157" s="5" t="s">
+        <v>471</v>
+      </c>
+      <c r="E157" s="5" t="s">
+        <v>472</v>
+      </c>
+      <c r="F157" s="5" t="s">
+        <v>473</v>
+      </c>
+      <c r="G157" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="H157" s="5"/>
+    </row>
+    <row r="158" spans="1:8" ht="32" customHeight="1">
+      <c r="A158" s="6" t="s">
+        <v>506</v>
+      </c>
+      <c r="B158" s="5" t="s">
+        <v>474</v>
+      </c>
+      <c r="C158" s="5">
+        <v>24</v>
+      </c>
+      <c r="D158" s="5" t="s">
+        <v>475</v>
+      </c>
+      <c r="E158" s="5" t="s">
+        <v>472</v>
+      </c>
+      <c r="F158" s="5" t="s">
+        <v>476</v>
+      </c>
+      <c r="G158" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="H158" s="5"/>
+    </row>
+    <row r="159" spans="1:8" ht="32" customHeight="1">
+      <c r="A159" s="6" t="s">
+        <v>506</v>
+      </c>
+      <c r="B159" s="5" t="s">
+        <v>477</v>
+      </c>
+      <c r="C159" s="5">
+        <v>2</v>
+      </c>
+      <c r="D159" s="5" t="s">
+        <v>478</v>
+      </c>
+      <c r="E159" s="5" t="s">
+        <v>479</v>
+      </c>
+      <c r="F159" s="5" t="s">
+        <v>480</v>
+      </c>
+      <c r="G159" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="H159" s="5" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="160" spans="1:8" ht="32" customHeight="1">
+      <c r="A160" s="6" t="s">
+        <v>506</v>
+      </c>
+      <c r="B160" s="5" t="s">
         <v>518</v>
       </c>
-      <c r="C153" s="5">
-        <v>1</v>
-      </c>
-      <c r="D153" s="5" t="s">
+      <c r="C160" s="5">
+        <v>1</v>
+      </c>
+      <c r="D160" s="5" t="s">
         <v>519</v>
       </c>
-      <c r="E153" s="5" t="s">
+      <c r="E160" s="5" t="s">
         <v>516</v>
       </c>
-      <c r="F153" s="5" t="s">
+      <c r="F160" s="5" t="s">
         <v>517</v>
       </c>
-      <c r="G153" s="5"/>
-      <c r="H153" s="5"/>
-    </row>
-    <row r="154" spans="1:8" s="10" customFormat="1" ht="32" customHeight="1">
-      <c r="A154" s="11" t="s">
+      <c r="G160" s="5"/>
+      <c r="H160" s="5"/>
+    </row>
+    <row r="161" spans="1:8" s="10" customFormat="1" ht="32" customHeight="1">
+      <c r="A161" s="11" t="s">
         <v>506</v>
       </c>
-      <c r="B154" s="9" t="s">
+      <c r="B161" s="9" t="s">
         <v>522</v>
       </c>
-      <c r="C154" s="9"/>
-      <c r="D154" s="9" t="s">
+      <c r="C161" s="9"/>
+      <c r="D161" s="9" t="s">
         <v>520</v>
       </c>
-      <c r="E154" s="9" t="s">
+      <c r="E161" s="9" t="s">
         <v>512</v>
       </c>
-      <c r="F154" s="9" t="s">
+      <c r="F161" s="9" t="s">
         <v>521</v>
       </c>
-      <c r="G154" s="9" t="s">
+      <c r="G161" s="9" t="s">
         <v>524</v>
       </c>
-      <c r="H154" s="9"/>
-    </row>
-    <row r="155" spans="1:8" s="14" customFormat="1" ht="32" customHeight="1">
-      <c r="A155" s="12" t="s">
+      <c r="H161" s="9"/>
+    </row>
+    <row r="162" spans="1:8" s="14" customFormat="1" ht="32" customHeight="1">
+      <c r="A162" s="12" t="s">
         <v>506</v>
       </c>
-      <c r="B155" s="13" t="s">
+      <c r="B162" s="13" t="s">
         <v>523</v>
       </c>
-      <c r="C155" s="13"/>
-      <c r="D155" s="13" t="s">
+      <c r="C162" s="13"/>
+      <c r="D162" s="13" t="s">
         <v>78</v>
       </c>
-      <c r="E155" s="13"/>
-      <c r="F155" s="13"/>
-      <c r="G155" s="9" t="s">
+      <c r="E162" s="13"/>
+      <c r="F162" s="13"/>
+      <c r="G162" s="9" t="s">
         <v>515</v>
       </c>
-      <c r="H155" s="13"/>
-    </row>
-    <row r="156" spans="1:8" s="14" customFormat="1" ht="32" customHeight="1">
-      <c r="A156" s="12" t="s">
+      <c r="H162" s="13"/>
+    </row>
+    <row r="163" spans="1:8" s="14" customFormat="1" ht="32" customHeight="1">
+      <c r="A163" s="12" t="s">
         <v>506</v>
       </c>
-      <c r="B156" s="13" t="s">
+      <c r="B163" s="13" t="s">
         <v>513</v>
       </c>
-      <c r="C156" s="13"/>
-      <c r="D156" s="13" t="s">
+      <c r="C163" s="13"/>
+      <c r="D163" s="13" t="s">
         <v>514</v>
       </c>
-      <c r="E156" s="13" t="s">
+      <c r="E163" s="13" t="s">
         <v>512</v>
       </c>
-      <c r="F156" s="13"/>
-      <c r="G156" s="13"/>
-      <c r="H156" s="13"/>
-    </row>
-    <row r="157" spans="1:8" s="14" customFormat="1" ht="32" customHeight="1">
-      <c r="A157" s="12" t="s">
+      <c r="F163" s="13"/>
+      <c r="G163" s="13"/>
+      <c r="H163" s="13"/>
+    </row>
+    <row r="164" spans="1:8" s="14" customFormat="1" ht="32" customHeight="1">
+      <c r="A164" s="12" t="s">
         <v>509</v>
       </c>
-      <c r="B157" s="13" t="s">
+      <c r="B164" s="13" t="s">
         <v>509</v>
       </c>
-      <c r="C157" s="13"/>
-      <c r="D157" s="13" t="s">
+      <c r="C164" s="13"/>
+      <c r="D164" s="13" t="s">
         <v>510</v>
       </c>
-      <c r="E157" s="13" t="s">
+      <c r="E164" s="13" t="s">
         <v>510</v>
       </c>
-      <c r="F157" s="13"/>
-      <c r="G157" s="13"/>
-      <c r="H157" s="13"/>
-    </row>
-    <row r="158" spans="1:8" s="10" customFormat="1" ht="32" customHeight="1">
-      <c r="A158" s="8" t="s">
+      <c r="F164" s="13"/>
+      <c r="G164" s="13"/>
+      <c r="H164" s="13"/>
+    </row>
+    <row r="165" spans="1:8" s="10" customFormat="1" ht="32" customHeight="1">
+      <c r="A165" s="8" t="s">
         <v>507</v>
       </c>
-      <c r="B158" s="9" t="s">
+      <c r="B165" s="9" t="s">
         <v>507</v>
       </c>
-      <c r="C158" s="9"/>
-      <c r="D158" s="9" t="s">
+      <c r="C165" s="9"/>
+      <c r="D165" s="9" t="s">
         <v>508</v>
       </c>
-      <c r="E158" s="9"/>
-      <c r="F158" s="9"/>
-      <c r="G158" s="9"/>
-      <c r="H158" s="9"/>
-    </row>
-    <row r="159" spans="1:8" ht="32" customHeight="1">
-      <c r="A159" s="7" t="s">
+      <c r="E165" s="9"/>
+      <c r="F165" s="9"/>
+      <c r="G165" s="9"/>
+      <c r="H165" s="9"/>
+    </row>
+    <row r="166" spans="1:8" ht="32" customHeight="1">
+      <c r="A166" s="7" t="s">
         <v>501</v>
       </c>
-      <c r="B159" s="7" t="s">
+      <c r="B166" s="7" t="s">
         <v>481</v>
       </c>
-      <c r="C159" s="7">
+      <c r="C166" s="7">
         <v>256</v>
       </c>
-      <c r="D159" s="7" t="s">
+      <c r="D166" s="7" t="s">
         <v>482</v>
       </c>
-      <c r="E159" s="7" t="s">
+      <c r="E166" s="7" t="s">
         <v>256</v>
       </c>
-      <c r="F159" s="7" t="s">
+      <c r="F166" s="7" t="s">
         <v>483</v>
       </c>
-      <c r="G159" s="7" t="s">
+      <c r="G166" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="H159" s="7"/>
-    </row>
-    <row r="160" spans="1:8" ht="32" customHeight="1">
-      <c r="A160" s="5" t="s">
+      <c r="H166" s="7"/>
+    </row>
+    <row r="167" spans="1:8" ht="32" customHeight="1">
+      <c r="A167" s="5" t="s">
         <v>501</v>
       </c>
-      <c r="B160" s="5" t="s">
+      <c r="B167" s="5" t="s">
         <v>484</v>
       </c>
-      <c r="C160" s="5">
+      <c r="C167" s="5">
         <v>2048</v>
       </c>
-      <c r="D160" s="5" t="s">
+      <c r="D167" s="5" t="s">
         <v>485</v>
       </c>
-      <c r="E160" s="5" t="s">
+      <c r="E167" s="5" t="s">
         <v>256</v>
       </c>
-      <c r="F160" s="5" t="s">
+      <c r="F167" s="5" t="s">
         <v>486</v>
       </c>
-      <c r="G160" s="5" t="s">
+      <c r="G167" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="H160" s="5"/>
-    </row>
-    <row r="161" spans="1:8" ht="32" customHeight="1">
-      <c r="A161" s="5" t="s">
+      <c r="H167" s="5"/>
+    </row>
+    <row r="168" spans="1:8" ht="32" customHeight="1">
+      <c r="A168" s="5" t="s">
         <v>501</v>
       </c>
-      <c r="B161" s="5" t="s">
+      <c r="B168" s="5" t="s">
         <v>502</v>
       </c>
-      <c r="C161" s="5">
+      <c r="C168" s="5">
         <v>256</v>
       </c>
-      <c r="D161" s="5" t="s">
+      <c r="D168" s="5" t="s">
         <v>511</v>
       </c>
-      <c r="E161" s="5" t="s">
+      <c r="E168" s="5" t="s">
         <v>512</v>
       </c>
-      <c r="F161" s="5"/>
-      <c r="G161" s="5"/>
-      <c r="H161" s="5"/>
-    </row>
-    <row r="162" spans="1:8" ht="32" customHeight="1">
-      <c r="A162" s="5" t="s">
+      <c r="F168" s="5"/>
+      <c r="G168" s="5"/>
+      <c r="H168" s="5"/>
+    </row>
+    <row r="169" spans="1:8" ht="32" customHeight="1">
+      <c r="A169" s="5" t="s">
         <v>503</v>
       </c>
-      <c r="B162" s="5" t="s">
+      <c r="B169" s="5" t="s">
         <v>503</v>
       </c>
-      <c r="C162" s="5">
+      <c r="C169" s="5">
         <v>4096</v>
       </c>
-      <c r="D162" s="5" t="s">
+      <c r="D169" s="5" t="s">
         <v>504</v>
       </c>
-      <c r="E162" s="5" t="s">
+      <c r="E169" s="5" t="s">
         <v>505</v>
       </c>
-      <c r="F162" s="5"/>
-      <c r="G162" s="5"/>
-      <c r="H162" s="5"/>
+      <c r="F169" s="5"/>
+      <c r="G169" s="5"/>
+      <c r="H169" s="5"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H160" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:H167" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.25" right="0.25" top="0.35" bottom="0.35" header="0.15" footer="0.15"/>
-  <pageSetup paperSize="11" scale="94" fitToHeight="0" orientation="landscape"/>
+  <pageSetup paperSize="11" scale="87" fitToHeight="0" orientation="landscape"/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>

</xml_diff>